<commit_message>
Started a new project in UPI analysis
</commit_message>
<xml_diff>
--- a/ms-excel practice lessons/Lesson No.12 - Paste special & GoTo Special/GOTO SPEICAL.xlsx
+++ b/ms-excel practice lessons/Lesson No.12 - Paste special & GoTo Special/GOTO SPEICAL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/80e58288fa9e0496/Desktop/MS-EXCEL/ms-excel practice lessons/Lesson No.12 - Paste special ^0 GoTo Special/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{618AD7B1-94A9-405E-91E9-A924FF63E719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72A5BB25-F630-443A-BFAD-95ED27B1909A}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="13_ncr:1_{618AD7B1-94A9-405E-91E9-A924FF63E719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8E02BBB-FFFF-4ED3-AED9-FAF635870C1F}"/>
   <bookViews>
-    <workbookView xWindow="732" yWindow="576" windowWidth="22128" windowHeight="13104" tabRatio="774" xr2:uid="{F3C24E79-9FB6-42BA-B8FC-ECC72FDF0E5E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="774" xr2:uid="{F3C24E79-9FB6-42BA-B8FC-ECC72FDF0E5E}"/>
   </bookViews>
   <sheets>
     <sheet name="BLANKS" sheetId="4" r:id="rId1"/>
@@ -102,7 +102,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="58">
   <si>
     <t>S. No.</t>
   </si>
@@ -261,6 +261,21 @@
   </si>
   <si>
     <t>MANAGER</t>
+  </si>
+  <si>
+    <t>Phone NO.</t>
+  </si>
+  <si>
+    <t>Lower case Desg</t>
+  </si>
+  <si>
+    <t>This sheet is being formatted on the basis of these two</t>
+  </si>
+  <si>
+    <t>1. Formatted on the basis of name starting with 'A'</t>
+  </si>
+  <si>
+    <t>2.  Formatted on the basis of salary &gt;= 15000</t>
   </si>
 </sst>
 </file>
@@ -270,7 +285,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -312,8 +327,15 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -338,8 +360,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -386,12 +420,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -411,12 +454,37 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="5">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -426,6 +494,27 @@
       <font>
         <color rgb="FF9C0006"/>
       </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -438,6 +527,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -738,7 +831,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D25AFB37-0545-4CAB-ABB0-E3FAC3CB5237}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
@@ -751,326 +844,413 @@
     <col min="8" max="8" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.44140625" customWidth="1"/>
     <col min="10" max="10" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="17" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J1" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="K1" s="18" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="4">
-        <v>15000</v>
-      </c>
-      <c r="F2" s="7">
+      <c r="E2" s="19">
+        <v>14000</v>
+      </c>
+      <c r="F2" s="20">
         <f>E2*20%</f>
-        <v>3000</v>
-      </c>
-      <c r="G2" s="3" t="b">
+        <v>2800</v>
+      </c>
+      <c r="G2" s="2" t="b">
         <f>AND(D2="MIS EXECUTIVE")</f>
         <v>1</v>
       </c>
-      <c r="H2" s="3" t="str">
+      <c r="H2" s="2" t="str">
         <f>UPPER(B2)</f>
         <v>ARUN</v>
       </c>
-      <c r="I2" t="str" cm="1">
+      <c r="I2" s="8" t="str" cm="1">
         <f t="array" ref="I2:J2">LOWER(C2:D2)</f>
         <v>tcs 1</v>
       </c>
-      <c r="J2" t="str">
+      <c r="J2" s="8" t="str">
         <v>mis executive</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K2" s="8">
+        <v>8033115308</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="19">
         <v>15000</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="20">
         <f t="shared" ref="F3:F9" si="0">E3*20%</f>
         <v>3000</v>
       </c>
-      <c r="G3" s="3" t="b">
+      <c r="G3" s="2" t="b">
         <f t="shared" ref="G3:G9" si="1">AND(D3="MIS EXECUTIVE")</f>
         <v>0</v>
       </c>
-      <c r="H3" s="3" t="str">
+      <c r="H3" s="2" t="str">
         <f t="shared" ref="H3:H8" si="2">UPPER(B3)</f>
         <v>TARUN</v>
       </c>
-      <c r="I3" t="str" cm="1">
+      <c r="I3" s="8" t="str" cm="1">
         <f t="array" ref="I3:J3">LOWER(C3:D3)</f>
         <v>tcs 2</v>
       </c>
-      <c r="J3" t="str">
+      <c r="J3" s="8" t="str">
         <v>consultant</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K3" s="8">
+        <v>9817393259</v>
+      </c>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
+      <c r="Q3" s="23"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="19">
         <v>12000</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="20">
         <f t="shared" si="0"/>
         <v>2400</v>
       </c>
-      <c r="G4" s="3" t="b">
+      <c r="G4" s="2" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H4" s="3" t="str">
+      <c r="H4" s="2" t="str">
         <f t="shared" si="2"/>
         <v>VARUN</v>
       </c>
-      <c r="I4" t="str" cm="1">
+      <c r="I4" s="8" t="str" cm="1">
         <f t="array" ref="I4:J4">LOWER(C4:D4)</f>
         <v>tcs 3</v>
       </c>
-      <c r="J4" t="str">
+      <c r="J4" s="8" t="str">
         <v>accounts executive</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K4" s="8">
+        <v>9126160741</v>
+      </c>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="23"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="19">
         <v>12000</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="20">
         <f t="shared" si="0"/>
         <v>2400</v>
       </c>
-      <c r="G5" s="3" t="b">
+      <c r="G5" s="2" t="b">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="H5" s="3" t="str">
+      <c r="H5" s="2" t="str">
         <f t="shared" si="2"/>
         <v>VIKAS</v>
       </c>
-      <c r="I5" t="str" cm="1">
+      <c r="I5" s="8" t="str" cm="1">
         <f t="array" ref="I5:J5">LOWER(C5:D5)</f>
         <v>tcs 4</v>
       </c>
-      <c r="J5" t="str">
+      <c r="J5" s="8" t="str">
         <v>mis executive</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K5" s="8">
+        <v>8192357871</v>
+      </c>
+      <c r="M5" s="23"/>
+      <c r="N5" s="23"/>
+      <c r="O5" s="23"/>
+      <c r="P5" s="23"/>
+      <c r="Q5" s="23"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="19">
         <v>12000</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="20">
         <f t="shared" si="0"/>
         <v>2400</v>
       </c>
-      <c r="G6" s="3" t="b">
+      <c r="G6" s="2" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H6" s="3" t="str">
+      <c r="H6" s="2" t="str">
         <f t="shared" si="2"/>
         <v>LALIT</v>
       </c>
-      <c r="I6" t="str" cm="1">
+      <c r="I6" s="8" t="str" cm="1">
         <f t="array" ref="I6:J6">LOWER(C6:D6)</f>
         <v>tcs 6</v>
       </c>
-      <c r="J6" t="str">
+      <c r="J6" s="8" t="str">
         <v>accounts executive</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K6" s="8">
+        <v>7056027093</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>7</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="19">
         <v>12000</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="20">
         <f t="shared" si="0"/>
         <v>2400</v>
       </c>
-      <c r="G7" s="3" t="b">
+      <c r="G7" s="2" t="b">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="H7" s="3" t="str">
+      <c r="H7" s="2" t="str">
         <f t="shared" si="2"/>
         <v>RAJU</v>
       </c>
-      <c r="I7" t="str" cm="1">
+      <c r="I7" s="8" t="str" cm="1">
         <f t="array" ref="I7:J7">LOWER(C7:D7)</f>
         <v>tcs 7</v>
       </c>
-      <c r="J7" t="str">
+      <c r="J7" s="8" t="str">
         <v>mis executive</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K7" s="8">
+        <v>9473340191</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>8</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="19">
         <v>15000</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="20">
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
-      <c r="G8" s="3" t="b">
+      <c r="G8" s="2" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H8" s="3" t="str">
+      <c r="H8" s="2" t="str">
         <f t="shared" si="2"/>
         <v>VAIBHAV</v>
       </c>
-      <c r="I8" t="str" cm="1">
+      <c r="I8" s="8" t="str" cm="1">
         <f t="array" ref="I8:J8">LOWER(C8:D8)</f>
         <v>tcs 8</v>
       </c>
-      <c r="J8" t="str">
+      <c r="J8" s="8" t="str">
         <v>consultant</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K8" s="8">
+        <v>8413774294</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>10</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="19">
         <v>75000</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="20">
         <f t="shared" si="0"/>
         <v>15000</v>
       </c>
-      <c r="G9" s="3" t="b">
+      <c r="G9" s="2" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H9" s="3" t="str">
+      <c r="H9" s="2" t="str">
         <f>UPPER(B9)</f>
         <v>SAGAR</v>
       </c>
-      <c r="I9" t="str" cm="1">
+      <c r="I9" s="8" t="str" cm="1">
         <f t="array" ref="I9:J9">LOWER(C9:D9)</f>
         <v>tcs 10</v>
       </c>
-      <c r="J9" t="str">
+      <c r="J9" s="8" t="str">
         <v>manager</v>
       </c>
+      <c r="K9" s="8">
+        <v>7931233167</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="C13" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="C14" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="C15" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="C14:G14"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A2:K9">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>LEFT($B2,1) ="A"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="2">
+      <formula>$E2 &gt;= 15000</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>